<commit_message>
Embed the six product photos as in-cell images
Place each cut-out PNG into column H with Excel's "place in cell" format
rather than as a floating shape, as the form asks for. That format keeps
the image behind a richValue reference chain, so the new entries are
appended to metadata.xml, rdrichvalue.xml and richValueRel.xml and the
two example images the form ships with (vm=1, 2) stay untouched.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013PR57qgwoN4kM429aZRbXL
</commit_message>
<xml_diff>
--- a/biteki-bestcosme/【つるりんちょ。】美的2027年1月号・美的MEN「下半期ベストコスメ」リサーチアンケート.xlsx
+++ b/biteki-bestcosme/【つるりんちょ。】美的2027年1月号・美的MEN「下半期ベストコスメ」リサーチアンケート.xlsx
@@ -40,7 +40,7 @@
   <metadataTypes count="1">
     <metadataType name="XLRICHVALUE" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1"/>
   </metadataTypes>
-  <futureMetadata name="XLRICHVALUE" count="2">
+  <futureMetadata name="XLRICHVALUE" count="8">
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
@@ -55,13 +55,73 @@
         </ext>
       </extLst>
     </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="2"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="3"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="4"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="5"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="6"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="7"/>
+        </ext>
+      </extLst>
+    </bk>
   </futureMetadata>
-  <valueMetadata count="2">
+  <valueMetadata count="8">
     <bk>
       <rc t="1" v="0"/>
     </bk>
     <bk>
       <rc t="1" v="1"/>
+    </bk>
+    <bk>
+      <rc t="1" v="2"/>
+    </bk>
+    <bk>
+      <rc t="1" v="3"/>
+    </bk>
+    <bk>
+      <rc t="1" v="4"/>
+    </bk>
+    <bk>
+      <rc t="1" v="5"/>
+    </bk>
+    <bk>
+      <rc t="1" v="6"/>
+    </bk>
+    <bk>
+      <rc t="1" v="7"/>
     </bk>
   </valueMetadata>
 </metadata>
@@ -2151,13 +2211,37 @@
 </file>
 
 <file path=xl/richData/rdrichvalue.xml><?xml version="1.0" encoding="utf-8"?>
-<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="2">
+<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="8">
   <rv s="0">
     <v>0</v>
     <v>5</v>
   </rv>
   <rv s="0">
     <v>1</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>2</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>3</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>4</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>5</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>6</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>7</v>
     <v>5</v>
   </rv>
 </rvData>
@@ -2176,6 +2260,12 @@
 <richValueRels xmlns="http://schemas.microsoft.com/office/spreadsheetml/2022/richvaluerel" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <rel r:id="rId1"/>
   <rel r:id="rId2"/>
+  <rel r:id="rId3"/>
+  <rel r:id="rId4"/>
+  <rel r:id="rId5"/>
+  <rel r:id="rId6"/>
+  <rel r:id="rId7"/>
+  <rel r:id="rId8"/>
 </richValueRels>
 </file>
 
@@ -3490,7 +3580,9 @@
           <t xml:space="preserve">400mL</t>
         </is>
       </c>
-      <c r="H62" s="53"/>
+      <c r="H62" s="53" t="e" vm="3">
+        <v>#VALUE!</v>
+      </c>
       <c r="I62" s="54">
         <v>46204</v>
       </c>
@@ -3536,7 +3628,9 @@
           <t xml:space="preserve">380g</t>
         </is>
       </c>
-      <c r="H63" s="43"/>
+      <c r="H63" s="43" t="e" vm="4">
+        <v>#VALUE!</v>
+      </c>
       <c r="I63" s="44">
         <v>46204</v>
       </c>
@@ -3582,7 +3676,9 @@
           <t xml:space="preserve">400mL</t>
         </is>
       </c>
-      <c r="H64" s="43"/>
+      <c r="H64" s="43" t="e" vm="5">
+        <v>#VALUE!</v>
+      </c>
       <c r="I64" s="44">
         <v>46204</v>
       </c>
@@ -3628,7 +3724,9 @@
           <t xml:space="preserve">380g</t>
         </is>
       </c>
-      <c r="H65" s="43"/>
+      <c r="H65" s="43" t="e" vm="6">
+        <v>#VALUE!</v>
+      </c>
       <c r="I65" s="44">
         <v>46204</v>
       </c>
@@ -3674,7 +3772,9 @@
           <t xml:space="preserve">380g</t>
         </is>
       </c>
-      <c r="H66" s="43"/>
+      <c r="H66" s="43" t="e" vm="7">
+        <v>#VALUE!</v>
+      </c>
       <c r="I66" s="44">
         <v>46204</v>
       </c>
@@ -3720,7 +3820,9 @@
           <t xml:space="preserve">400mL</t>
         </is>
       </c>
-      <c r="H67" s="43"/>
+      <c r="H67" s="43" t="e" vm="8">
+        <v>#VALUE!</v>
+      </c>
       <c r="I67" s="44">
         <v>46204</v>
       </c>

</xml_diff>